<commit_message>
docs(order-history/order-management): extend sibling story docs to implementation-status format
Bring the 17 non-13.2 story feasibility docs (.md + .xlsx) up to the extended
implementation-status format per STORY_DOC_FORMAT_UPDATES.md, additively.

- 13.1: delivered via SBE-1146 (Story 13.2's shipped GET /orders)
- 13.3 + 24.1-24.15: honest "Not started - analysis only" status

Each .md gains an Implementation line, an Implementation Status section, and
status-tagged Open Questions (+ Deferred Work where a req is blocked/deferred).
Each .xlsx gains an Impl Status column, Status/Resolution Open-Questions columns,
an Implementation Status sheet, and Overview impl rows.
</commit_message>
<xml_diff>
--- a/order_history/13.1-order-history/13.1 - Order History.xlsx
+++ b/order_history/13.1-order-history/13.1 - Order History.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Endpoints" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Open Questions" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Cross-Epic Dependencies" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Implementation Status" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requirements'!$A$1:$K$7</definedName>
@@ -112,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -150,6 +151,10 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -515,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -654,6 +659,54 @@
       </c>
       <c r="B13" s="8" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Delivered via SBE-1146 (Story 13.2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Impl Branch</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>feature/SBE-1146-order-listing-table</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Impl Commits</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09bce5f, fc429bd</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>#272</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -667,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -681,6 +734,7 @@
     <col width="48" customWidth="1" min="9" max="9"/>
     <col width="62" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -739,6 +793,11 @@
           <t>Confluence</t>
         </is>
       </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>Impl Status (2026-07-01)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -792,6 +851,11 @@
           <t>Open §Order History → Story 13.1</t>
         </is>
       </c>
+      <c r="L2" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146, via 13.2)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -845,6 +909,11 @@
           <t>Open §Order History → Story 13.1</t>
         </is>
       </c>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146, via 13.2)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -898,6 +967,11 @@
           <t>Open §Order History → Story 13.1</t>
         </is>
       </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146, via 13.2)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -951,6 +1025,11 @@
           <t>Open §Order History → Story 13.1</t>
         </is>
       </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146, via 13.2)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1008,6 +1087,11 @@
           <t>Open §Order History → Story 13.1</t>
         </is>
       </c>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>✅ Done (SBE-1146, via 13.2)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1059,6 +1143,11 @@
       <c r="K7" s="11" t="inlineStr">
         <is>
           <t>Open §Order History → Story 13.1</t>
+        </is>
+      </c>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>Out of Scope — 13.2</t>
         </is>
       </c>
     </row>
@@ -1157,11 +1246,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="120" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1175,6 +1266,16 @@
           <t>Open Question</t>
         </is>
       </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Resolution / Decision</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -1183,6 +1284,16 @@
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Should abandoned 'pending' orders (a pending row is created at place-order time before the Stripe redirect; if the user backs out it stays pending forever) be shown in Order History, or excluded? The existing PPL order-history endpoint deliberately excludes them and shows only terminal/active states, but 13.1's mandate to show 'current' orders plus the sibling 'pay' action imply active payable orders (e.g. partially_paid split plans) must appear — confirm whether never-paid abandoned-checkout orders are included or filtered out.</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>Open — for team discussion</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>Current direction (2026-07-01): mirrors Story 13.2 — the shipped GET /orders INCLUDES pending rows so in-flight/current orders surface (consistent with 13.1's past-AND-current mandate and the Pay action). Flagged for team confirmation because it also surfaces never-paid abandoned-checkout rows; team to confirm keep / age-filter / exclude abandoned-checkout pending (single where predicate if it changes).</t>
         </is>
       </c>
     </row>
@@ -1234,4 +1345,106 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Shipped (SBE-1146, via 13.2)</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Story 13.1 owns no independent endpoint; all in-scope requirements are delivered by building Story 13.2's shipped GET /orders listing (branch feature/SBE-1146-order-listing-table, commits 09bce5f + fc429bd, PR #272 → dev, Swagger tag Orders). Covers 13.1-a,b,c,d,e (empty state folded into 13.2 as 13.2-m).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Remaining — none</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>No independent work remains — completing Story 13.2 completes this story.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Open decision — pending orders</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Whether abandoned pending orders appear in the listing; mirrored from 13.2's direction (currently SHIPPED as included). Team to confirm keep / age-filter / exclude abandoned-checkout pending (single where predicate if it changes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Dependency — 13.2</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>GET /orders listing endpoint owned by Story 13.2 (Order Listing Table) — the single canonical route this container story rides on; per-row actions/columns defined there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Out of scope — 13.1-f</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Order-level actions (View/Invoice/Pay) delegated to Story 13.2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Out of API scope</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Front-end page / row-to-detail / action wiring.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(order-history): reconcile 13.1/13.2 docs to product-only listing (SBE-1621)
Update the Order History feasibility + implementation docs (md and xlsx
mirrors) to match the shipped SBE-1621 change: GET /orders is now scoped to
order_type = product, so subscription/ppl_addon orders no longer appear in
the exhibitor Order History listing (they remain on /ppl/orders).

- 13.2 Implementation Plan: Gate Contract, Design Decision D5, What/tests/
  verification updated; added Revision Log v1.2.
- 13.2 Order Listing Table (md + xlsx): Open Q#1 marked SUPERSEDED,
  pending-inclusion + Q#2 decisions clarified.
- 13.1 Order History (md + xlsx): 13.1-a/13.1-d completeness reconciled.
- Feasibility Summary xlsx: Endpoint Catalog GET /orders purpose.

Key nuance preserved: SBE-1621 re-applies only the order_type = product
filter, NOT the pending-exclusion of the earlier reverted variant, so
pending product orders still list. Confluence story update is tracked
separately by SBE-1618 (BA-owned).
</commit_message>
<xml_diff>
--- a/order_history/13.1-order-history/13.1 - Order History.xlsx
+++ b/order_history/13.1-order-history/13.1 - Order History.xlsx
@@ -827,7 +827,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>No aggregate (all-order-type) order-history controller exists yet, so the endpoint is net-new — but a structurally identical Order-History list already ships for PPL (company-scoped Order.findMany, created_at desc, paginated, search), and a second list reference (purchased-booths) exists. The new endpoint reuses the same pattern but drops the order_type/status narrowing so it spans all purchases. The Order model is written by live checkout flows.</t>
+          <t>No aggregate (all-order-type) order-history controller exists yet, so the endpoint is net-new — but a structurally identical Order-History list already ships for PPL (company-scoped Order.findMany, created_at desc, paginated, search), and a second list reference (purchased-booths) exists. The new endpoint reuses the same pattern, scoped to order_type = product (SBE-1621) across all statuses incl. pending; subscription/ppl_addon remain on /ppl/orders. The Order model is written by live checkout flows.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>All order types (subscription, ppl_addon, product) exist and are written by live flows, and Order.status is actively transitioned by the Stripe webhook to completed, partially_paid, failed, canceled (plus pending at creation). The new endpoint simply omits the narrowing the two reference lists apply (purchased-booths→product/completed; ppl→subscription+ppl_addon/terminal). Note: the 'refunded' OrderStatus enum value is NOT written to Order by any production write-path (only paymentTransaction.status and read-only display mapping use it), but this does not gate the requirement — the listing shows whatever statuses exist and refunds aren't yet a checkout outcome.</t>
+          <t>All order types (subscription, ppl_addon, product) exist and are written by live flows, and Order.status is actively transitioned by the Stripe webhook to completed, partially_paid, failed, canceled (plus pending at creation). The new endpoint applies only the order_type = product type filter (SBE-1621 — matching purchased-booths' type predicate) but keeps ALL statuses incl. pending (it does not apply purchased-booths' completed/terminal status filter); subscription/ppl_addon orders are served by /ppl/orders. Note: the 'refunded' OrderStatus enum value is NOT written to Order by any production write-path (only paymentTransaction.status and read-only display mapping use it), but this does not gate the requirement — the listing shows whatever statuses exist and refunds aren't yet a checkout outcome.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">

</xml_diff>